<commit_message>
new storage nodes and connections
</commit_message>
<xml_diff>
--- a/mes_north_sea/clean_data/new_technologies/NewTechnologies_2040.xlsx
+++ b/mes_north_sea/clean_data/new_technologies/NewTechnologies_2040.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/Key-Infrastructure-North-Sea-CodeAndData/mes_north_sea/clean_data/new_technologies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5817A44-D7F0-5648-B775-D427B5454F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EF4A96-354F-EF47-9CA6-64870252A183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
+    <workbookView xWindow="1280" yWindow="500" windowWidth="27520" windowHeight="15980" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
   </bookViews>
   <sheets>
     <sheet name="NewTechnologies" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1270" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="127">
   <si>
     <t>Electrolyser_PEM_offshore</t>
   </si>
@@ -396,9 +396,21 @@
     <t>Offshore_Wind, DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
   </si>
   <si>
+    <t>DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
+  </si>
+  <si>
+    <t>DAC_Adsorption_offshore, HeatPump_AirSourced_offshore, PermanentStorage_CO2_simple</t>
+  </si>
+  <si>
+    <t>Offshore_Wind, DAC_Adsorption_offshore, HeatPump_AirSourced_offshore, PermanentStorage_CO2_simple</t>
+  </si>
+  <si>
     <t>DK_ST1</t>
   </si>
   <si>
+    <t>New_CO2_Storage_2040</t>
+  </si>
+  <si>
     <t>NO_ST2</t>
   </si>
   <si>
@@ -408,20 +420,14 @@
     <t>NO_ST1</t>
   </si>
   <si>
-    <t>New_CO2_Storage_2040</t>
-  </si>
-  <si>
-    <t>PermanentStorage_CO2_simple</t>
-  </si>
-  <si>
-    <t>DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
+    <t>PermanentStorage_CO2_simple, DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -435,6 +441,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -444,7 +457,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -452,12 +465,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1164,6 +1190,9 @@
       <c r="B9" t="s">
         <v>2</v>
       </c>
+      <c r="C9" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="E9" t="s">
         <v>45</v>
       </c>
@@ -1252,6 +1281,9 @@
       <c r="B11" t="s">
         <v>2</v>
       </c>
+      <c r="C11" t="s">
+        <v>126</v>
+      </c>
       <c r="E11" t="s">
         <v>45</v>
       </c>
@@ -1296,6 +1328,9 @@
       <c r="B12" t="s">
         <v>2</v>
       </c>
+      <c r="C12" t="s">
+        <v>126</v>
+      </c>
       <c r="E12" t="s">
         <v>45</v>
       </c>
@@ -1340,6 +1375,9 @@
       <c r="B13" t="s">
         <v>2</v>
       </c>
+      <c r="C13" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="E13" t="s">
         <v>45</v>
       </c>
@@ -1385,7 +1423,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E14" t="s">
         <v>45</v>
@@ -1432,7 +1470,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
         <v>45</v>
@@ -1479,7 +1517,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E16" t="s">
         <v>45</v>
@@ -1526,7 +1564,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E17" t="s">
         <v>45</v>
@@ -1573,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E18" t="s">
         <v>45</v>
@@ -1620,7 +1658,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E19" t="s">
         <v>45</v>
@@ -1667,7 +1705,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E20" t="s">
         <v>45</v>
@@ -1714,7 +1752,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E21" t="s">
         <v>45</v>
@@ -1761,7 +1799,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
@@ -1808,7 +1846,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E23" t="s">
         <v>45</v>
@@ -3764,7 +3802,7 @@
         <v>64</v>
       </c>
       <c r="C47" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -3930,7 +3968,7 @@
         <v>64</v>
       </c>
       <c r="C49" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D49" t="s">
         <v>49</v>
@@ -4013,7 +4051,7 @@
         <v>64</v>
       </c>
       <c r="C50" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D50" t="s">
         <v>49</v>
@@ -4179,7 +4217,7 @@
         <v>64</v>
       </c>
       <c r="C52" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D52" t="s">
         <v>49</v>
@@ -4262,7 +4300,7 @@
         <v>64</v>
       </c>
       <c r="C53" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D53" t="s">
         <v>49</v>
@@ -4588,46 +4626,46 @@
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>118</v>
-      </c>
-      <c r="B57" t="s">
+        <v>121</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>122</v>
       </c>
       <c r="C57" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>119</v>
-      </c>
-      <c r="B58" t="s">
+        <v>123</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C58" t="s">
-        <v>123</v>
+      <c r="C58" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="59" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>120</v>
-      </c>
-      <c r="B59" t="s">
+        <v>124</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C59" t="s">
-        <v>123</v>
+      <c r="C59" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>121</v>
-      </c>
-      <c r="B60" t="s">
+        <v>125</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C60" t="s">
-        <v>123</v>
+      <c r="C60" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated hp techno-economic parameters
</commit_message>
<xml_diff>
--- a/mes_north_sea/clean_data/new_technologies/NewTechnologies_2040.xlsx
+++ b/mes_north_sea/clean_data/new_technologies/NewTechnologies_2040.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/Key-Infrastructure-North-Sea-CodeAndData/mes_north_sea/clean_data/new_technologies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EF4A96-354F-EF47-9CA6-64870252A183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFA0F17-B616-C141-8340-014254F50626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1280" yWindow="500" windowWidth="27520" windowHeight="15980" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
   </bookViews>
   <sheets>
     <sheet name="NewTechnologies" sheetId="1" r:id="rId1"/>
@@ -393,18 +393,6 @@
     <t>Onshore_Wind, PV, DAC_Adsorption_onshore, HeatPump_AirSourced_onshore</t>
   </si>
   <si>
-    <t>Offshore_Wind, DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
-  </si>
-  <si>
-    <t>DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
-  </si>
-  <si>
-    <t>DAC_Adsorption_offshore, HeatPump_AirSourced_offshore, PermanentStorage_CO2_simple</t>
-  </si>
-  <si>
-    <t>Offshore_Wind, DAC_Adsorption_offshore, HeatPump_AirSourced_offshore, PermanentStorage_CO2_simple</t>
-  </si>
-  <si>
     <t>DK_ST1</t>
   </si>
   <si>
@@ -420,7 +408,19 @@
     <t>NO_ST1</t>
   </si>
   <si>
-    <t>PermanentStorage_CO2_simple, DAC_Adsorption_offshore, HeatPump_AirSourced_offshore</t>
+    <t>PermanentStorage_CO2_simple, DAC_Adsorption_offshore, HeatPump_SeaWaterSourced</t>
+  </si>
+  <si>
+    <t>DAC_Adsorption_offshore, HeatPump_SeaWaterSourced</t>
+  </si>
+  <si>
+    <t>DAC_Adsorption_offshore, HeatPump_SeaWaterSourced, PermanentStorage_CO2_simple</t>
+  </si>
+  <si>
+    <t>Offshore_Wind, DAC_Adsorption_offshore, HeatPump_SeaWaterSourced</t>
+  </si>
+  <si>
+    <t>Offshore_Wind, DAC_Adsorption_offshore, HeatPump_SeaWaterSourced, PermanentStorage_CO2_simple</t>
   </si>
 </sst>
 </file>
@@ -1191,7 +1191,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E9" t="s">
         <v>45</v>
@@ -1282,7 +1282,7 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
         <v>45</v>
@@ -1329,7 +1329,7 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E12" t="s">
         <v>45</v>
@@ -1376,7 +1376,7 @@
         <v>2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E13" t="s">
         <v>45</v>
@@ -1423,7 +1423,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E14" t="s">
         <v>45</v>
@@ -1470,7 +1470,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E15" t="s">
         <v>45</v>
@@ -1517,7 +1517,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E16" t="s">
         <v>45</v>
@@ -1564,7 +1564,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E17" t="s">
         <v>45</v>
@@ -1611,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E18" t="s">
         <v>45</v>
@@ -1658,7 +1658,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E19" t="s">
         <v>45</v>
@@ -1705,7 +1705,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E20" t="s">
         <v>45</v>
@@ -1752,7 +1752,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E21" t="s">
         <v>45</v>
@@ -1799,7 +1799,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
@@ -1846,7 +1846,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E23" t="s">
         <v>45</v>
@@ -3221,7 +3221,7 @@
         <v>64</v>
       </c>
       <c r="C40" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D40" t="s">
         <v>49</v>
@@ -3304,7 +3304,7 @@
         <v>64</v>
       </c>
       <c r="C41" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D41" t="s">
         <v>49</v>
@@ -3387,7 +3387,7 @@
         <v>64</v>
       </c>
       <c r="C42" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D42" t="s">
         <v>49</v>
@@ -3470,7 +3470,7 @@
         <v>64</v>
       </c>
       <c r="C43" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D43" t="s">
         <v>49</v>
@@ -3553,7 +3553,7 @@
         <v>64</v>
       </c>
       <c r="C44" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D44" t="s">
         <v>49</v>
@@ -3636,7 +3636,7 @@
         <v>64</v>
       </c>
       <c r="C45" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D45" t="s">
         <v>49</v>
@@ -3719,7 +3719,7 @@
         <v>64</v>
       </c>
       <c r="C46" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D46" t="s">
         <v>49</v>
@@ -3802,7 +3802,7 @@
         <v>64</v>
       </c>
       <c r="C47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -3885,7 +3885,7 @@
         <v>64</v>
       </c>
       <c r="C48" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D48" t="s">
         <v>49</v>
@@ -3968,7 +3968,7 @@
         <v>64</v>
       </c>
       <c r="C49" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D49" t="s">
         <v>49</v>
@@ -4051,7 +4051,7 @@
         <v>64</v>
       </c>
       <c r="C50" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D50" t="s">
         <v>49</v>
@@ -4134,7 +4134,7 @@
         <v>64</v>
       </c>
       <c r="C51" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D51" t="s">
         <v>49</v>
@@ -4217,7 +4217,7 @@
         <v>64</v>
       </c>
       <c r="C52" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D52" t="s">
         <v>49</v>
@@ -4300,7 +4300,7 @@
         <v>64</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D53" t="s">
         <v>49</v>
@@ -4383,7 +4383,7 @@
         <v>64</v>
       </c>
       <c r="C54" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D54" t="s">
         <v>49</v>
@@ -4466,7 +4466,7 @@
         <v>64</v>
       </c>
       <c r="C55" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D55" t="s">
         <v>49</v>
@@ -4549,7 +4549,7 @@
         <v>64</v>
       </c>
       <c r="C56" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D56" t="s">
         <v>49</v>
@@ -4626,46 +4626,46 @@
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C57" t="s">
         <v>122</v>
-      </c>
-      <c r="C57" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B58" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="59" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B59" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>